<commit_message>
add heatsinks 2X QDM2 from Thorlabs
</commit_message>
<xml_diff>
--- a/Benchtop-2024(default-version)/parts-list/Benchtop-partslist-latest.xlsx
+++ b/Benchtop-2024(default-version)/parts-list/Benchtop-partslist-latest.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Nikita\Documents\GitHub\mesoSPIM-bt-hardware\Benchtop-2024(default-version)\parts-list\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF9CBF7F-39C7-49A0-A92E-0E0E9D300304}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44385B0C-13D5-4A7E-A0F5-E4854459FF61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7200" yWindow="1320" windowWidth="34560" windowHeight="18600" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="10752" yWindow="2388" windowWidth="30156" windowHeight="21264" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Main" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1024" uniqueCount="626">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1024" uniqueCount="625">
   <si>
     <t xml:space="preserve">Part # </t>
   </si>
@@ -1838,18 +1838,6 @@
     <t>already accounted for, see AB90H, 5x, above</t>
   </si>
   <si>
-    <t>Heat sink for galvo driver, 100x75x25 mm or similar</t>
-  </si>
-  <si>
-    <t>2x-servo-boards-QS-series</t>
-  </si>
-  <si>
-    <t>See /galvo-assembly/heatsink-servo-boards</t>
-  </si>
-  <si>
-    <t>Blank heatsink from Mouser or elsewhere</t>
-  </si>
-  <si>
     <t>RD-PDT-S-to-M4-bolts-Base-H10mm</t>
   </si>
   <si>
@@ -1981,6 +1969,15 @@
   </si>
   <si>
     <t>Ø12.7 mm Optical Post, SS, M4 Setscrew, M6 Tap, L = 75 mm</t>
+  </si>
+  <si>
+    <t>QDM2</t>
+  </si>
+  <si>
+    <t>Heatsink and Mount for QG4, QG5, QS15, QS20, QS30, and QS45 Galvanometer System Servo Drivers</t>
+  </si>
+  <si>
+    <t>For DIY heat sink, see /galvo-assembly/heatsink-servo-boards</t>
   </si>
 </sst>
 </file>
@@ -2871,13 +2868,13 @@
     </row>
     <row r="8" spans="1:9" s="87" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="87" t="s">
-        <v>616</v>
+        <v>612</v>
       </c>
       <c r="B8" s="87" t="s">
-        <v>617</v>
+        <v>613</v>
       </c>
       <c r="C8" s="87" t="s">
-        <v>618</v>
+        <v>614</v>
       </c>
       <c r="D8" s="87">
         <v>2</v>
@@ -2893,12 +2890,12 @@
         <v>34</v>
       </c>
       <c r="I8" s="87" t="s">
-        <v>619</v>
+        <v>615</v>
       </c>
     </row>
     <row r="9" spans="1:9" s="89" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A9" s="89" t="s">
-        <v>615</v>
+        <v>611</v>
       </c>
       <c r="B9" s="89" t="s">
         <v>161</v>
@@ -2920,7 +2917,7 @@
         <v>34</v>
       </c>
       <c r="I9" s="19" t="s">
-        <v>620</v>
+        <v>616</v>
       </c>
     </row>
     <row r="10" spans="1:9" s="6" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.3">
@@ -2932,7 +2929,7 @@
     </row>
     <row r="11" spans="1:9" s="28" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A11" s="28" t="s">
-        <v>592</v>
+        <v>588</v>
       </c>
       <c r="B11" s="28" t="s">
         <v>18</v>
@@ -3070,7 +3067,7 @@
     </row>
     <row r="16" spans="1:9" s="28" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A16" s="28" t="s">
-        <v>593</v>
+        <v>589</v>
       </c>
       <c r="B16" s="28" t="s">
         <v>18</v>
@@ -3235,13 +3232,13 @@
     </row>
     <row r="23" spans="1:9" s="28" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A23" s="53" t="s">
-        <v>594</v>
+        <v>590</v>
       </c>
       <c r="B23" s="28" t="s">
         <v>18</v>
       </c>
       <c r="C23" s="28" t="s">
-        <v>595</v>
+        <v>591</v>
       </c>
       <c r="D23" s="28">
         <v>0</v>
@@ -3452,7 +3449,7 @@
         <v>233</v>
       </c>
       <c r="I32" s="3" t="s">
-        <v>590</v>
+        <v>586</v>
       </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.25">
@@ -3479,7 +3476,7 @@
         <v>233</v>
       </c>
       <c r="I33" s="3" t="s">
-        <v>591</v>
+        <v>587</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
@@ -3565,7 +3562,7 @@
     </row>
     <row r="37" spans="1:9" s="4" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A37" s="82" t="s">
-        <v>587</v>
+        <v>583</v>
       </c>
       <c r="B37" s="10" t="s">
         <v>205</v>
@@ -3584,7 +3581,7 @@
         <v>10</v>
       </c>
       <c r="I37" s="4" t="s">
-        <v>588</v>
+        <v>584</v>
       </c>
     </row>
     <row r="38" spans="1:9" s="12" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.3">
@@ -3596,77 +3593,77 @@
     </row>
     <row r="39" spans="1:9" s="12" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A39" s="86" t="s">
-        <v>613</v>
+        <v>609</v>
       </c>
       <c r="E39" s="59"/>
       <c r="F39" s="59"/>
     </row>
     <row r="40" spans="1:9" s="84" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A40" s="83" t="s">
-        <v>599</v>
+        <v>595</v>
       </c>
       <c r="B40" s="83" t="s">
-        <v>604</v>
+        <v>600</v>
       </c>
       <c r="E40" s="85"/>
       <c r="F40" s="85"/>
     </row>
     <row r="41" spans="1:9" s="84" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A41" s="83" t="s">
-        <v>600</v>
+        <v>596</v>
       </c>
       <c r="B41" s="83" t="s">
-        <v>605</v>
+        <v>601</v>
       </c>
       <c r="E41" s="85"/>
       <c r="F41" s="85"/>
     </row>
     <row r="42" spans="1:9" s="84" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A42" s="83" t="s">
-        <v>606</v>
+        <v>602</v>
       </c>
       <c r="B42" s="83" t="s">
-        <v>607</v>
+        <v>603</v>
       </c>
       <c r="E42" s="85"/>
       <c r="F42" s="85"/>
     </row>
     <row r="43" spans="1:9" s="84" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A43" s="83" t="s">
-        <v>608</v>
+        <v>604</v>
       </c>
       <c r="B43" s="83" t="s">
-        <v>603</v>
+        <v>599</v>
       </c>
       <c r="E43" s="85"/>
       <c r="F43" s="85"/>
     </row>
     <row r="44" spans="1:9" s="84" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A44" s="83" t="s">
-        <v>601</v>
+        <v>597</v>
       </c>
       <c r="B44" s="83" t="s">
-        <v>602</v>
+        <v>598</v>
       </c>
       <c r="E44" s="85"/>
       <c r="F44" s="85"/>
     </row>
     <row r="45" spans="1:9" s="84" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A45" s="83" t="s">
-        <v>611</v>
+        <v>607</v>
       </c>
       <c r="B45" s="83" t="s">
-        <v>612</v>
+        <v>608</v>
       </c>
       <c r="E45" s="85"/>
       <c r="F45" s="85"/>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A46" s="3" t="s">
-        <v>609</v>
+        <v>605</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>610</v>
+        <v>606</v>
       </c>
     </row>
     <row r="47" spans="1:9" s="6" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.3">
@@ -4521,7 +4518,7 @@
         <v>203</v>
       </c>
       <c r="I76" s="4" t="s">
-        <v>589</v>
+        <v>585</v>
       </c>
     </row>
     <row r="77" spans="1:10" x14ac:dyDescent="0.25">
@@ -4586,13 +4583,13 @@
     </row>
     <row r="79" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A79" s="9" t="s">
-        <v>621</v>
+        <v>617</v>
       </c>
       <c r="B79" s="3" t="s">
         <v>54</v>
       </c>
       <c r="C79" s="9" t="s">
-        <v>622</v>
+        <v>618</v>
       </c>
       <c r="D79" s="3">
         <v>2</v>
@@ -4608,18 +4605,18 @@
         <v>34</v>
       </c>
       <c r="H79" s="3" t="s">
-        <v>623</v>
+        <v>619</v>
       </c>
     </row>
     <row r="80" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A80" s="9" t="s">
-        <v>624</v>
+        <v>620</v>
       </c>
       <c r="B80" s="3" t="s">
         <v>54</v>
       </c>
       <c r="C80" s="9" t="s">
-        <v>625</v>
+        <v>621</v>
       </c>
       <c r="D80" s="3">
         <v>2</v>
@@ -4635,7 +4632,7 @@
         <v>34</v>
       </c>
       <c r="H80" s="3" t="s">
-        <v>623</v>
+        <v>619</v>
       </c>
     </row>
     <row r="81" spans="1:9" s="23" customFormat="1" x14ac:dyDescent="0.25">
@@ -4995,34 +4992,34 @@
         <v>526</v>
       </c>
     </row>
-    <row r="93" spans="1:9" s="4" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A93" s="10" t="s">
-        <v>584</v>
-      </c>
-      <c r="B93" s="4" t="s">
-        <v>586</v>
-      </c>
-      <c r="C93" s="10" t="s">
-        <v>583</v>
-      </c>
-      <c r="D93" s="4">
-        <v>1</v>
-      </c>
-      <c r="E93" s="60">
-        <v>10</v>
-      </c>
-      <c r="F93" s="58">
+    <row r="93" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A93" s="9" t="s">
+        <v>622</v>
+      </c>
+      <c r="B93" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="C93" s="9" t="s">
+        <v>623</v>
+      </c>
+      <c r="D93" s="3">
+        <v>2</v>
+      </c>
+      <c r="E93" s="57">
+        <v>181</v>
+      </c>
+      <c r="F93" s="55">
         <f t="shared" si="6"/>
-        <v>10</v>
-      </c>
-      <c r="G93" s="4" t="s">
+        <v>362</v>
+      </c>
+      <c r="G93" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="H93" s="4" t="s">
+      <c r="H93" s="3" t="s">
         <v>200</v>
       </c>
-      <c r="I93" s="4" t="s">
-        <v>585</v>
+      <c r="I93" s="3" t="s">
+        <v>624</v>
       </c>
     </row>
     <row r="94" spans="1:9" x14ac:dyDescent="0.25">
@@ -5895,7 +5892,7 @@
         <v>44</v>
       </c>
       <c r="I133" s="3" t="s">
-        <v>614</v>
+        <v>610</v>
       </c>
     </row>
     <row r="134" spans="1:9" x14ac:dyDescent="0.25">
@@ -6825,7 +6822,7 @@
       </c>
       <c r="F182" s="50">
         <f>SUM(F3:F180)</f>
-        <v>136295.75149920007</v>
+        <v>136647.75149920007</v>
       </c>
       <c r="G182" s="3" t="s">
         <v>438</v>
@@ -6964,7 +6961,7 @@
     </row>
     <row r="201" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A201" s="3" t="s">
-        <v>587</v>
+        <v>583</v>
       </c>
       <c r="B201" s="3">
         <v>1</v>
@@ -7155,7 +7152,7 @@
     </row>
     <row r="6" spans="1:9" s="28" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
       <c r="B6" s="28" t="s">
-        <v>596</v>
+        <v>592</v>
       </c>
     </row>
     <row r="7" spans="1:9" s="6" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.3">
@@ -7188,7 +7185,7 @@
     </row>
     <row r="9" spans="1:9" s="28" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
       <c r="B9" s="28" t="s">
-        <v>597</v>
+        <v>593</v>
       </c>
     </row>
     <row r="10" spans="1:9" s="28" customFormat="1" ht="13.2" x14ac:dyDescent="0.25"/>
@@ -7749,7 +7746,7 @@
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B39" t="s">
-        <v>598</v>
+        <v>594</v>
       </c>
     </row>
     <row r="42" spans="1:9" s="7" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">

</xml_diff>